<commit_message>
Auto update P2P 2026-02-03 09:26
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -491,15 +491,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -583,7 +587,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -596,11 +600,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -624,11 +624,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -667,7 +663,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -695,12 +691,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -713,11 +709,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -727,7 +719,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -759,12 +751,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -791,12 +783,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -823,12 +815,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -855,12 +847,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Damien Vincent</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -887,12 +879,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Damien Vincent</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -919,12 +911,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -942,11 +934,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -955,12 +943,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -978,11 +966,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
@@ -991,12 +975,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1014,12 +998,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1027,12 +1011,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Carla Gallén</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1050,12 +1034,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1063,12 +1047,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1171,12 +1155,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Carla Gallén</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1207,12 +1191,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1243,12 +1227,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1271,7 +1255,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1279,12 +1267,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1399,7 +1387,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1439,7 +1427,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1472,23 +1460,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1516,18 +1500,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>José Messias Garcia da Silva Ferreira</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1571,12 +1551,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1615,12 +1595,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1659,12 +1639,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1703,12 +1683,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1736,23 +1716,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1785,22 +1765,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1828,11 +1804,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1843,12 +1815,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1891,12 +1863,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1939,12 +1911,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1987,7 +1959,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Núria Paredes Garcia</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2035,7 +2007,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2083,7 +2055,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2131,7 +2103,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2179,7 +2151,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Trinidad Piedra Clemente</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2227,7 +2199,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Trinidad Piedra Clemente</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2270,12 +2242,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2318,17 +2294,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Albert Roqué Morera</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2375,12 +2355,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Alicia Ripoll Bau</t>
+          <t>Cristina Melgosa Ramos</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2427,12 +2407,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2479,12 +2459,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Lumerli Oviedo Abreu</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2531,12 +2511,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Alicia Ripoll Bau</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2583,12 +2563,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Marc Puigventós</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2635,12 +2615,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2687,12 +2667,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Núria Paredes Garcia</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2739,7 +2719,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Susi anandam Subramanian</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2791,12 +2771,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Lumerli Oviedo Abreu</t>
+          <t>Elian Daghoum Dorado</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2843,12 +2823,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Elian Daghoum Dorado</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2887,6 +2867,58 @@
         </is>
       </c>
       <c r="J61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-04 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1011,12 +1011,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Carla Gallén</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1047,12 +1047,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Carla Gallén</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1191,12 +1191,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1219,7 +1219,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -1227,12 +1231,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1267,7 +1271,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1347,7 +1351,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1387,7 +1391,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1427,12 +1431,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1467,12 +1471,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1551,12 +1555,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1584,23 +1588,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1639,12 +1643,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1771,7 +1775,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1804,7 +1808,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1815,7 +1823,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1863,12 +1871,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1911,7 +1919,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1959,7 +1967,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2007,7 +2015,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2055,7 +2063,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2103,12 +2111,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2151,7 +2159,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2199,7 +2207,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Trinidad Piedra Clemente</t>
+          <t>Núria Paredes Garcia</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2251,12 +2259,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2303,12 +2311,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2355,12 +2363,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Marc Puigventós</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2407,12 +2415,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Alicia Ripoll Bau</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2511,12 +2519,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Alicia Ripoll Bau</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2563,12 +2571,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2615,12 +2623,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Cristina Melgosa Ramos</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2667,12 +2675,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Núria Paredes Garcia</t>
+          <t>Albert Roqué Morera</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2719,7 +2727,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Elian Daghoum Dorado</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2771,12 +2779,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Elian Daghoum Dorado</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2823,12 +2831,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2867,58 +2875,6 @@
         </is>
       </c>
       <c r="J61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-05 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,7 +515,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -539,12 +539,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -563,12 +563,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -587,12 +587,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -611,12 +611,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -635,12 +635,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -691,12 +691,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -719,12 +719,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -751,12 +751,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -783,7 +783,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -815,12 +815,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -847,12 +847,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -879,12 +879,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Damien Vincent</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -911,7 +911,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -943,12 +943,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -967,7 +967,11 @@
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -975,7 +979,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -998,12 +1002,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1011,12 +1015,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Franco Nicolas Ruiz Miras</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1024,11 +1028,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1039,7 +1039,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1047,12 +1051,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Carla Gallén</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1083,12 +1087,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Carla Gallén</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1119,12 +1123,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Franco Nicolas Ruiz Miras</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1132,7 +1136,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1143,11 +1151,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1155,12 +1159,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1183,7 +1187,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -1191,12 +1199,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1231,7 +1239,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1271,7 +1279,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1351,7 +1359,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1391,7 +1399,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1431,12 +1439,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1471,12 +1479,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1504,19 +1512,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1555,12 +1567,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1588,12 +1600,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1643,12 +1655,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>José Messias Garcia da Silva Ferreira</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1687,12 +1699,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1720,23 +1732,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1769,18 +1781,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1823,12 +1839,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1871,12 +1887,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1919,7 +1935,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1967,7 +1983,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2015,12 +2031,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2063,7 +2079,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2111,12 +2127,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2159,7 +2175,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Núria Paredes Garcia</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2202,17 +2218,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Núria Paredes Garcia</t>
+          <t>Marc Puigventós</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2311,7 +2331,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Elian Daghoum Dorado</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2363,7 +2383,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Alicia Ripoll Bau</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2415,12 +2435,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Alicia Ripoll Bau</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2467,7 +2487,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Lumerli Oviedo Abreu</t>
+          <t>Albert Roqué Morera</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2519,7 +2539,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Cristina Melgosa Ramos</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2623,7 +2643,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2675,7 +2695,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Lumerli Oviedo Abreu</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2727,7 +2747,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Elian Daghoum Dorado</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2779,7 +2799,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2823,58 +2843,6 @@
         </is>
       </c>
       <c r="J60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-06 09:23
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,7 +515,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -563,7 +563,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -587,12 +587,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -611,12 +611,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -635,12 +635,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -691,12 +691,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -719,12 +719,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -751,12 +751,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -783,7 +783,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -815,12 +815,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -847,12 +847,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -879,12 +879,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -911,12 +911,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -934,7 +934,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -1015,12 +1019,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Franco Nicolas Ruiz Miras</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1028,7 +1032,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1039,11 +1047,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1051,7 +1055,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1079,7 +1083,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1087,12 +1095,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Carla Gallén</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1115,7 +1123,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1123,12 +1135,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1151,7 +1163,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1159,12 +1175,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1182,24 +1198,24 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1239,12 +1255,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1279,7 +1295,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1319,12 +1335,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1342,24 +1358,24 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1399,12 +1415,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1432,19 +1448,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1472,19 +1492,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>José Messias Garcia da Silva Ferreira</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1523,12 +1547,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1567,12 +1591,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1600,23 +1624,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1655,7 +1679,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1693,18 +1717,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1732,7 +1760,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1743,12 +1775,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1791,12 +1823,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1839,7 +1871,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1882,17 +1914,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1930,17 +1966,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1978,17 +2018,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Marc Puigventós</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2026,17 +2070,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2074,17 +2122,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2122,17 +2174,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Elian Daghoum Dorado</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2170,17 +2226,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Núria Paredes Garcia</t>
+          <t>Alicia Ripoll Bau</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2227,12 +2287,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Núria Paredes Garcia</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2279,12 +2339,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2331,12 +2391,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Elian Daghoum Dorado</t>
+          <t>Lumerli Oviedo Abreu</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2383,12 +2443,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Alicia Ripoll Bau</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2435,12 +2495,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2487,7 +2547,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Cristina Melgosa Ramos</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2539,7 +2599,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Albert Roqué Morera</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2591,12 +2651,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2643,12 +2703,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2695,12 +2755,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Lumerli Oviedo Abreu</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2739,110 +2799,6 @@
         </is>
       </c>
       <c r="J58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Lorena Gonzalez</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-09 12:07
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -491,19 +491,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -515,7 +511,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -523,11 +519,7 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -539,19 +531,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -563,19 +551,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -587,12 +571,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -635,7 +619,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -648,11 +632,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -663,12 +643,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -676,11 +656,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -691,7 +667,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -704,11 +680,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -719,7 +691,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -737,11 +709,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -751,12 +719,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -769,11 +737,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -783,7 +747,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -801,11 +765,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -815,12 +775,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -847,12 +807,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -879,12 +839,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -911,12 +871,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -934,11 +894,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -947,12 +903,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -971,11 +927,7 @@
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -983,12 +935,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1006,11 +958,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
@@ -1019,12 +967,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1055,12 +1003,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1078,11 +1026,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1095,7 +1039,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1123,11 +1067,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1135,12 +1075,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1163,11 +1103,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1175,7 +1111,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1198,29 +1134,29 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1255,12 +1191,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1295,12 +1231,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1335,12 +1271,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1375,7 +1311,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1415,12 +1351,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1438,28 +1374,24 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1492,23 +1424,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1536,23 +1464,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1580,18 +1504,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1624,23 +1548,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>José Messias Garcia da Silva Ferreira</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1679,12 +1603,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1717,17 +1641,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1765,17 +1685,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1813,22 +1729,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1871,12 +1783,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1914,21 +1826,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1966,16 +1874,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2018,21 +1922,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2079,7 +1979,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2131,12 +2031,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2183,12 +2083,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Elian Daghoum Dorado</t>
+          <t>Albert Roqué Morera</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2287,12 +2187,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Núria Paredes Garcia</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2339,7 +2239,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Núria Paredes Garcia</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2391,12 +2291,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Lumerli Oviedo Abreu</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2443,12 +2343,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2495,12 +2395,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2547,12 +2447,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2599,7 +2499,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Lumerli Oviedo Abreu</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2651,12 +2551,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2703,12 +2603,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2755,50 +2655,154 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>Cristina Melgosa Ramos</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Marc Puigventós</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-10 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -839,7 +839,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -871,12 +871,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -935,12 +935,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -958,7 +958,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
@@ -1003,7 +1007,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1026,12 +1030,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1039,12 +1043,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1062,12 +1066,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1075,12 +1079,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1151,12 +1155,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1174,24 +1178,24 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1271,7 +1275,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1311,7 +1315,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1351,12 +1355,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1374,24 +1378,24 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1431,7 +1435,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1559,12 +1563,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1603,12 +1607,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>José Messias Garcia da Silva Ferreira</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1735,12 +1739,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1783,12 +1787,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1879,12 +1883,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1927,7 +1931,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1979,7 +1983,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2031,7 +2035,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2083,12 +2087,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Marc Puigventós</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2187,12 +2191,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Núria Paredes Garcia</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2239,12 +2243,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Núria Paredes Garcia</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2291,12 +2295,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2343,7 +2347,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2395,7 +2399,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2447,12 +2451,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Lumerli Oviedo Abreu</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2499,7 +2503,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Lumerli Oviedo Abreu</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2551,7 +2555,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2603,7 +2607,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Cristina Melgosa Ramos</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2655,7 +2659,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Albert Roqué Morera</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2707,7 +2711,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-02-11 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,7 +511,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -531,7 +531,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -551,12 +551,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -571,19 +571,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -595,7 +591,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -619,12 +615,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -643,12 +639,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -667,12 +663,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -680,7 +676,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -691,12 +691,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -775,7 +775,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -807,12 +807,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -839,12 +839,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -871,12 +871,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -894,7 +894,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -903,12 +907,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -926,7 +930,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
@@ -935,7 +943,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -971,12 +979,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -994,14 +1002,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1035,7 +1047,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1043,12 +1059,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1066,7 +1082,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1079,7 +1099,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1107,7 +1127,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1115,7 +1139,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1155,12 +1179,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1178,24 +1202,24 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1235,12 +1259,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1275,7 +1299,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1395,7 +1419,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1428,19 +1452,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1468,14 +1496,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1508,23 +1540,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1563,12 +1595,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1607,7 +1639,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1651,12 +1683,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1689,18 +1721,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1733,7 +1769,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1787,12 +1827,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1830,17 +1870,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1878,12 +1922,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1926,7 +1974,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1983,12 +2035,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Marc Puigventós</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2035,7 +2087,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2087,7 +2139,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>José Messias Garcia da Silva Ferreira</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2139,7 +2191,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Alicia Ripoll Bau</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2191,12 +2243,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Núria Paredes Garcia</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2243,7 +2295,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2295,12 +2347,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Alicia Ripoll Bau</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2347,7 +2399,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2399,12 +2451,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Albert Roqué Morera</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2451,7 +2503,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Lumerli Oviedo Abreu</t>
+          <t>Cristina Melgosa Ramos</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2503,7 +2555,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2555,7 +2607,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2607,7 +2659,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Lumerli Oviedo Abreu</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2659,12 +2711,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2711,12 +2763,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2755,58 +2807,6 @@
         </is>
       </c>
       <c r="J59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-12 11:09
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -531,7 +531,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -691,7 +691,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -719,12 +719,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -766,7 +766,11 @@
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -775,12 +779,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -807,12 +811,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -871,7 +875,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -907,12 +911,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -943,12 +947,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -979,12 +983,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1002,29 +1006,29 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1059,7 +1063,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1099,7 +1103,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1139,12 +1143,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1179,12 +1183,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1259,7 +1263,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1299,12 +1303,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Carla Gallén</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1339,12 +1343,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1379,12 +1383,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1412,14 +1416,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1442,23 +1450,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1507,12 +1515,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1551,12 +1559,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1595,7 +1603,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1639,12 +1647,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1683,12 +1691,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1721,22 +1729,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1779,12 +1783,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1827,7 +1831,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1879,12 +1883,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Marc Puigventós</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1931,7 +1935,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1983,7 +1987,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2035,12 +2039,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2087,12 +2091,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2139,12 +2143,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2347,12 +2351,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Alicia Ripoll Bau</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2399,12 +2403,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Alicia Ripoll Bau</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2451,12 +2455,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2503,7 +2507,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Albert Roqué Morera</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2555,7 +2559,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Cristina Melgosa Ramos</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2607,7 +2611,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2659,7 +2663,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Lumerli Oviedo Abreu</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2711,12 +2715,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Lumerli Oviedo Abreu</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2763,50 +2767,102 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>José Messias Garcia da Silva Ferreira</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-16 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -491,7 +491,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -531,7 +531,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -591,19 +591,15 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
@@ -615,12 +611,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -639,12 +635,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -663,12 +659,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -676,11 +672,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -691,12 +683,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -704,11 +696,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -719,12 +707,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -732,11 +720,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -747,7 +731,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>christopher rancel</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -760,17 +744,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -779,7 +755,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -792,16 +768,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -811,12 +779,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -829,11 +797,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -843,12 +807,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -861,11 +825,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -875,12 +835,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -893,16 +853,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -911,12 +863,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -934,11 +886,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
@@ -947,12 +895,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -965,11 +913,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>✅</t>
@@ -983,12 +927,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1006,16 +950,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1023,12 +959,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1046,16 +982,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1063,7 +991,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1091,11 +1019,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1103,12 +1027,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1131,11 +1055,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1143,12 +1063,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1171,11 +1091,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -1183,12 +1099,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1223,12 +1139,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1263,7 +1179,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1303,12 +1219,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Carla Gallén</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1343,12 +1259,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1383,7 +1299,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1416,18 +1332,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1450,33 +1362,29 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1504,23 +1412,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1548,23 +1452,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Carla Gallén</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1592,23 +1492,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1647,12 +1543,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1691,12 +1587,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1735,7 +1631,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1773,17 +1669,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1821,22 +1713,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1869,26 +1757,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1906,16 +1786,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1935,12 +1807,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1973,26 +1845,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2030,16 +1894,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2082,21 +1942,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2143,12 +1999,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2195,12 +2051,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2247,12 +2103,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2299,12 +2155,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2351,12 +2207,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>José Messias Garcia da Silva Ferreira</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2403,7 +2259,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Alicia Ripoll Bau</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2455,12 +2311,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2507,12 +2363,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2559,12 +2415,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2611,12 +2467,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2663,7 +2519,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Albert Roqué Morera</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2715,12 +2571,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Lumerli Oviedo Abreu</t>
+          <t>Alicia Ripoll Bau</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2767,12 +2623,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Cristina Melgosa Ramos</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2819,50 +2675,310 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>Laura Morales Guinart</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Ruben Serra Sanz</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Lumerli Oviedo Abreu</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Andre Mazurkiewitz</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Marc Puigventós</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-17 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,7 +471,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -531,12 +531,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -551,12 +551,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -571,7 +571,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -591,12 +591,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -611,7 +611,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -619,11 +619,7 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -635,7 +631,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -643,11 +639,7 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -659,19 +651,15 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -683,7 +671,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -691,11 +679,7 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -707,12 +691,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -731,12 +715,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>christopher rancel</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -755,12 +739,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -779,12 +763,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -792,11 +776,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
@@ -807,7 +787,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -820,11 +800,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
@@ -835,12 +811,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -863,12 +839,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -881,11 +857,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -895,12 +867,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -914,11 +886,7 @@
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
@@ -927,7 +895,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -959,12 +927,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -977,12 +945,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
@@ -991,7 +959,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1014,11 +982,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
@@ -1027,12 +991,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1050,11 +1014,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
@@ -1063,12 +1023,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1086,11 +1046,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
@@ -1099,12 +1055,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1127,11 +1083,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -1139,7 +1091,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1167,11 +1119,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1179,7 +1127,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1207,11 +1155,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -1219,7 +1163,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1259,7 +1203,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1299,12 +1243,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1339,12 +1283,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1379,7 +1323,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1419,12 +1363,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1459,12 +1403,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Carla Gallén</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1499,7 +1443,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1532,18 +1476,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1566,28 +1506,28 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1631,12 +1571,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1719,12 +1659,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1763,7 +1703,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1786,33 +1726,33 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1851,12 +1791,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1889,22 +1829,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1937,17 +1873,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1990,21 +1922,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2042,11 +1970,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2103,7 +2027,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2155,7 +2079,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2207,12 +2131,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Laura Soto Alsina</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2259,12 +2183,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2311,12 +2235,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2363,12 +2287,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>José Messias Garcia da Silva Ferreira</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2415,7 +2339,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2467,7 +2391,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2571,7 +2495,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Alicia Ripoll Bau</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2623,12 +2547,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2675,7 +2599,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Cristina Melgosa Ramos</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2727,12 +2651,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Alicia Ripoll Bau</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2779,7 +2703,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Lumerli Oviedo Abreu</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2831,7 +2755,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2883,12 +2807,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Lumerli Oviedo Abreu</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2935,50 +2859,154 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>Andre Mazurkiewitz</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Marc Puigventós</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-19 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -511,7 +511,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -531,12 +531,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -551,12 +551,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -571,12 +571,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -591,7 +591,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -611,12 +611,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -631,12 +631,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -651,12 +651,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -671,12 +671,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -691,19 +691,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -715,12 +711,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -739,12 +735,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -763,7 +759,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -787,7 +783,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -811,12 +807,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -867,12 +863,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -885,7 +881,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -895,12 +895,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -927,12 +927,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -945,12 +945,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
@@ -959,12 +959,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -991,12 +991,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1014,7 +1014,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
@@ -1023,7 +1027,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1046,7 +1050,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
@@ -1055,7 +1063,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1091,12 +1099,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1127,7 +1135,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1155,7 +1163,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -1163,7 +1175,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1203,7 +1215,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1243,12 +1255,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1283,12 +1295,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1323,12 +1335,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1363,12 +1375,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1403,7 +1415,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1443,7 +1455,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1483,7 +1495,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1506,33 +1518,33 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1571,12 +1583,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1615,7 +1627,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1659,7 +1671,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1703,12 +1715,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1791,12 +1803,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1829,18 +1841,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1863,18 +1879,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1927,7 +1947,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1970,12 +1990,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2027,7 +2051,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2079,12 +2103,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2131,7 +2155,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Laura Soto Alsina</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2235,7 +2259,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2287,12 +2311,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>José Messias Garcia da Silva Ferreira</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2339,7 +2363,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Marc Puigventós</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2391,7 +2415,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2443,7 +2467,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Albert Roqué Morera</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2495,12 +2519,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2547,7 +2571,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2599,12 +2623,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Cristina Melgosa Ramos</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2703,12 +2727,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2755,12 +2779,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2799,214 +2823,6 @@
         </is>
       </c>
       <c r="J63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Lumerli Oviedo Abreu</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Andre Mazurkiewitz</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Marc Puigventós</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-20 09:22
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -471,7 +471,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -531,12 +531,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -551,7 +551,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -591,12 +591,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -651,12 +651,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -671,7 +671,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -691,12 +691,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -711,7 +711,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -735,12 +735,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -759,7 +759,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -783,12 +783,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -895,7 +895,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -927,12 +927,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -959,12 +959,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -991,12 +991,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1027,7 +1027,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1063,12 +1063,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1335,12 +1335,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1455,12 +1455,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1671,7 +1671,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1715,12 +1715,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1753,7 +1753,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1797,18 +1801,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1831,11 +1839,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1846,17 +1850,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1879,7 +1887,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1890,16 +1902,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2051,12 +2059,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2103,12 +2111,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2259,12 +2267,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Marc Puigventós</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2311,12 +2319,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Lorena Gonzalez</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2363,12 +2371,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2415,12 +2423,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Laura Morales Guinart</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2467,12 +2475,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ruben Serra Sanz</t>
+          <t>Ismael Hernández</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2519,7 +2527,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Ruben Serra Sanz</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2571,7 +2579,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ismael Hernández</t>
+          <t>Ester Pinna</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2623,12 +2631,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Ester Pinna</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2675,7 +2683,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Alicia Ripoll Bau</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2727,7 +2735,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Alicia Ripoll Bau</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-02-23 15:48
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -531,12 +531,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -551,7 +551,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -571,12 +571,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -591,12 +591,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -611,7 +611,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -651,7 +651,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -671,12 +671,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -691,15 +691,19 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -711,7 +715,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -735,7 +739,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -759,12 +763,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -772,7 +776,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
@@ -783,7 +791,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -796,7 +804,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
@@ -807,7 +819,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -835,12 +847,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -863,12 +875,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -895,7 +907,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -927,12 +939,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -950,7 +962,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
@@ -982,7 +998,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
@@ -1027,7 +1047,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1063,12 +1083,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1099,12 +1119,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1215,7 +1235,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1255,7 +1275,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1295,7 +1315,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1335,7 +1355,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1415,7 +1435,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1495,7 +1515,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1539,12 +1559,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1583,12 +1603,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1627,7 +1647,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1665,18 +1685,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1699,28 +1723,32 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1763,12 +1791,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1811,12 +1839,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1839,7 +1867,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1850,11 +1882,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1907,7 +1935,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1955,7 +1983,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2007,12 +2035,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2059,12 +2087,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2111,7 +2139,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2215,7 +2243,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2267,7 +2295,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Marc Puigventós</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2319,12 +2347,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Lorena Gonzalez</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2371,12 +2399,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2423,12 +2451,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Laura Morales Guinart</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2467,370 +2495,6 @@
         </is>
       </c>
       <c r="J56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Ismael Hernández</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Ruben Serra Sanz</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Ester Pinna</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Andre Mazurkiewitz</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Andrey Ismagilov</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Alicia Ripoll Bau</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-02-25 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -591,12 +591,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -631,7 +631,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -651,7 +651,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -671,15 +671,19 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -1195,7 +1199,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1235,12 +1239,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1275,7 +1279,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1315,7 +1319,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1355,12 +1359,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1395,12 +1399,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1435,7 +1439,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1468,19 +1472,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1508,19 +1516,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1559,12 +1571,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1603,12 +1615,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-02-25 14:18
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -491,7 +491,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -511,7 +511,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -531,7 +531,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -539,7 +539,11 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -551,15 +555,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -571,15 +579,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
@@ -591,15 +603,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
@@ -611,15 +627,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -631,15 +651,19 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -660,7 +684,11 @@
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -671,7 +699,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -695,7 +723,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -719,7 +747,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -743,12 +771,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -756,7 +784,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
@@ -767,12 +799,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -795,12 +827,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -823,7 +855,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -879,7 +911,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -911,7 +943,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -943,12 +975,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -979,12 +1011,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1015,7 +1047,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1051,12 +1083,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1087,12 +1119,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1123,12 +1155,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1199,12 +1231,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1239,12 +1271,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1399,7 +1431,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1432,19 +1464,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1483,12 +1519,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1527,12 +1563,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1571,12 +1607,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1615,12 +1651,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1653,18 +1689,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1947,12 +1987,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1990,17 +2030,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2047,12 +2091,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2099,7 +2143,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2203,12 +2247,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2255,7 +2299,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2307,12 +2351,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2359,12 +2403,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2411,12 +2455,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-02-27 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -511,15 +511,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -531,7 +535,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -555,12 +559,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -579,7 +583,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -603,7 +607,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -611,12 +615,12 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -627,7 +631,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -651,12 +655,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -675,20 +679,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -699,12 +703,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -723,7 +727,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -747,7 +751,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -771,7 +775,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -799,12 +803,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -827,12 +831,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -845,7 +849,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -855,12 +863,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -873,7 +881,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -883,12 +895,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -901,7 +913,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -911,12 +927,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -943,12 +959,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -975,7 +991,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1011,7 +1027,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1047,12 +1063,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1083,12 +1099,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-03-05 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -535,12 +535,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -559,7 +559,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -583,20 +583,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -607,20 +607,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -631,12 +631,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -655,12 +655,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -679,12 +679,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -703,12 +703,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -821,7 +821,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -831,12 +835,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -863,12 +867,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -927,7 +931,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -959,7 +963,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -991,12 +995,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1063,12 +1067,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1099,12 +1103,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1171,12 +1175,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1207,7 +1211,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1247,12 +1251,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1287,12 +1291,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1367,12 +1371,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1407,12 +1411,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1447,7 +1451,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1491,12 +1495,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1535,12 +1539,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1579,7 +1583,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1623,12 +1627,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1661,18 +1665,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1695,11 +1703,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1710,7 +1714,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1763,12 +1771,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1791,7 +1799,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1802,16 +1814,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1849,22 +1857,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1907,12 +1915,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1955,12 +1963,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2003,12 +2011,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2055,7 +2063,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2107,12 +2115,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2159,7 +2167,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Telesforo Sol</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2211,12 +2219,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2263,12 +2271,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2315,7 +2323,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Margot Arroyo</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2367,12 +2375,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2419,12 +2427,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2471,12 +2479,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-03-06 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -559,12 +559,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -583,20 +583,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -607,7 +607,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -631,20 +631,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -655,12 +655,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -679,7 +679,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -703,12 +703,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -727,7 +727,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -751,7 +751,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -775,12 +775,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -793,7 +793,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -803,12 +807,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -835,12 +839,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -867,7 +871,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -899,12 +903,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -931,7 +935,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -963,12 +967,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -986,7 +990,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
@@ -995,12 +1003,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1031,12 +1039,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1067,7 +1075,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1139,12 +1147,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1157,17 +1165,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -1175,7 +1183,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1211,12 +1219,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1251,12 +1259,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1291,12 +1299,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1331,12 +1339,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1364,19 +1372,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1404,14 +1416,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1444,14 +1460,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1489,18 +1509,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1533,18 +1557,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1567,23 +1595,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1621,18 +1653,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1665,22 +1701,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1703,7 +1739,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1714,16 +1754,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1771,7 +1807,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1819,12 +1855,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1857,22 +1893,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1915,12 +1951,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1963,12 +1999,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2006,12 +2042,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2063,12 +2103,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Andrea Carozza</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2115,7 +2155,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2167,12 +2207,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Telesforo Sol</t>
+          <t>Andre Mazurkiewitz</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2219,12 +2259,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2323,7 +2363,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Margot Arroyo</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2375,7 +2415,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2427,7 +2467,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2471,110 +2511,6 @@
         </is>
       </c>
       <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Andrea Carozza</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-03-10 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,15 +491,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -511,12 +515,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -535,7 +539,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -559,20 +563,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -583,12 +587,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -607,7 +611,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -620,7 +624,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -631,15 +639,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>✅</t>
@@ -655,7 +667,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -668,7 +680,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -679,7 +695,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -692,7 +708,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -703,12 +723,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -716,8 +736,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -727,7 +755,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -740,8 +768,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -751,12 +787,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -764,8 +800,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -775,7 +819,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -807,12 +851,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -839,12 +883,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -871,12 +915,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -903,7 +947,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -935,7 +979,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -958,7 +1002,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
@@ -967,12 +1015,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -985,17 +1033,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1003,7 +1051,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1039,12 +1087,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1075,12 +1123,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1139,7 +1187,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -1147,12 +1199,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1165,7 +1217,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1183,12 +1239,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1211,7 +1267,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1219,7 +1279,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1292,14 +1352,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1332,7 +1396,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
     </row>
@@ -1383,12 +1451,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1421,13 +1489,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1465,18 +1537,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1615,12 +1691,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1663,7 +1739,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1701,22 +1777,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1759,12 +1835,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1797,22 +1873,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1855,7 +1931,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1903,12 +1979,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1951,12 +2027,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1999,12 +2075,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2051,12 +2127,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2103,7 +2179,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Andrea Carozza</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2155,12 +2231,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2259,12 +2335,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2311,12 +2387,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2363,7 +2439,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2415,12 +2491,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2459,58 +2535,6 @@
         </is>
       </c>
       <c r="J53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-03-11 09:40
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -883,12 +883,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -915,12 +915,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1159,12 +1159,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1199,12 +1199,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1239,12 +1239,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1279,12 +1279,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1312,7 +1312,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
     </row>
@@ -1691,12 +1695,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1739,7 +1743,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1787,7 +1791,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1825,17 +1829,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1873,22 +1877,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1931,12 +1935,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1974,12 +1978,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2022,12 +2030,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2070,17 +2082,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2127,7 +2143,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2179,12 +2195,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2231,7 +2247,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2439,7 +2455,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-03-12 09:28
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -563,7 +563,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -571,12 +571,12 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -587,12 +587,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -600,7 +600,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -611,7 +615,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -639,7 +643,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -667,7 +671,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -695,7 +699,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -713,7 +717,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -723,7 +731,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -755,12 +763,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -787,12 +795,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -819,12 +827,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -851,7 +859,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -915,7 +923,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -947,7 +955,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -979,12 +987,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1015,12 +1023,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1033,17 +1041,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1051,12 +1059,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1087,12 +1095,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1115,7 +1123,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1123,12 +1135,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1151,7 +1163,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1159,7 +1175,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1199,12 +1215,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1239,7 +1255,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1279,7 +1295,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1367,12 +1383,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1411,12 +1427,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-03-13 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -1255,12 +1255,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1288,19 +1288,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1339,7 +1343,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1383,12 +1387,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1427,12 +1431,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1855,12 +1859,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1903,12 +1907,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1946,17 +1950,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2003,7 +2011,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2055,12 +2063,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2107,12 +2115,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2159,7 +2167,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2211,7 +2219,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2263,12 +2271,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-03-13 09:50
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -491,7 +491,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -515,7 +515,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -539,12 +539,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -563,12 +563,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -699,12 +699,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -731,7 +731,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -763,12 +763,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -827,12 +827,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -859,7 +859,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -891,12 +891,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -923,12 +923,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1023,7 +1023,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1059,7 +1059,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1095,12 +1095,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1135,7 +1135,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1175,12 +1175,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1255,12 +1255,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1343,12 +1343,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1431,12 +1431,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1469,18 +1469,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1523,12 +1527,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1571,12 +1575,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1619,7 +1623,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1647,11 +1651,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1662,12 +1662,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1695,7 +1699,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1706,21 +1714,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2011,12 +2015,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2063,12 +2067,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-03-16 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,7 +471,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,7 +491,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -499,11 +499,7 @@
           <t>Joan</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
@@ -515,7 +511,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -523,11 +519,7 @@
           <t>Joan</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -539,19 +531,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
@@ -563,19 +551,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -587,24 +571,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -615,24 +591,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -643,7 +611,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -651,16 +619,8 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -671,12 +631,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -684,11 +644,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -699,12 +655,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -712,16 +668,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -731,12 +679,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -744,16 +692,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -763,12 +703,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,16 +716,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -795,7 +727,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -813,11 +745,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -827,12 +755,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -845,11 +773,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -859,12 +783,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -877,11 +801,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -891,12 +811,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -909,11 +829,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -923,12 +839,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -955,12 +871,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -987,12 +903,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1010,11 +926,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
@@ -1023,12 +935,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1046,11 +958,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
@@ -1059,12 +967,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1082,11 +990,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
@@ -1095,12 +999,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1118,16 +1022,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1135,7 +1031,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1158,16 +1054,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1175,12 +1063,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1198,16 +1086,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -1215,12 +1095,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1238,16 +1118,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -1255,7 +1127,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1283,28 +1155,20 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1327,23 +1191,15 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1371,28 +1227,20 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1420,23 +1268,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1464,27 +1308,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1512,22 +1348,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1560,22 +1388,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1613,22 +1433,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1651,32 +1467,28 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1709,22 +1521,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1757,22 +1565,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1815,12 +1619,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1853,12 +1657,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1911,7 +1715,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1954,21 +1758,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2006,21 +1806,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2043,11 +1839,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2067,12 +1859,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2110,21 +1902,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2157,11 +1945,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2171,12 +1955,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2214,21 +1998,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2266,21 +2046,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2327,7 +2103,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Andre Mazurkiewitz</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2379,12 +2155,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2431,12 +2207,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2483,12 +2259,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2535,50 +2311,362 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>Ramiro Aguilar Andrade</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Rossemary Castellanos</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Armando Aguilar Campos</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Vanessa Bujaldon Pellicer</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Ignacio Soldevilla</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-03-17 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -631,12 +631,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -655,7 +655,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -679,7 +679,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -703,12 +703,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -716,7 +716,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -727,12 +731,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -783,7 +787,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -903,7 +907,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -935,12 +939,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -967,7 +971,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -999,12 +1003,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1031,12 +1035,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1063,7 +1067,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1095,7 +1099,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Nicolás Aros</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1118,7 +1122,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
@@ -1127,12 +1135,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1163,7 +1171,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1199,12 +1207,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1235,12 +1243,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1275,12 +1283,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1315,12 +1323,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1355,12 +1363,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1395,7 +1403,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1483,12 +1491,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1527,12 +1535,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1571,12 +1579,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1619,12 +1627,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1667,7 +1675,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1715,7 +1723,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Federico Caruso Pérez</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1753,22 +1761,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1811,12 +1819,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1839,7 +1847,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1850,21 +1862,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1907,7 +1915,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1945,17 +1953,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2003,12 +2011,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2031,11 +2039,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2046,12 +2050,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2103,12 +2111,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2155,12 +2163,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2207,7 +2215,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2259,12 +2267,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2311,7 +2319,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2363,12 +2371,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Andrey Ismagilov</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2467,7 +2475,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2519,12 +2527,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2571,7 +2579,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-03-19 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -511,7 +511,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -531,7 +531,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -551,12 +551,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -571,12 +571,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -611,7 +611,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -703,7 +703,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -731,12 +731,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -787,7 +787,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -815,12 +815,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -843,12 +843,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -875,7 +875,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -907,7 +907,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -971,12 +971,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1003,12 +1003,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1035,12 +1035,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1067,12 +1067,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1090,7 +1090,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
@@ -1135,12 +1139,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1243,12 +1247,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1283,7 +1287,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1323,12 +1327,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1363,7 +1367,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1403,7 +1407,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1447,12 +1451,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1491,12 +1495,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1579,7 +1583,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1627,12 +1631,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1771,12 +1775,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1819,12 +1823,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1867,12 +1871,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1895,11 +1899,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1910,17 +1910,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2011,12 +2015,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2039,7 +2043,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H47" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2050,21 +2058,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2111,12 +2115,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Patricia Proniewska</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2163,12 +2167,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2215,12 +2219,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2267,7 +2271,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2319,7 +2323,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2423,7 +2427,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2579,7 +2583,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2631,7 +2635,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-03-23 11:54
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -531,12 +531,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -571,12 +571,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -591,12 +591,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -631,19 +631,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -655,7 +651,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Raúl Martínez</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -663,11 +659,7 @@
           <t>Joan</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -679,19 +671,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -703,7 +691,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -711,16 +699,8 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -731,7 +711,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -739,16 +719,8 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
@@ -759,24 +731,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Mohammad Gholinezhad</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
@@ -787,12 +751,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -800,11 +764,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
@@ -815,12 +775,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -828,11 +788,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
@@ -843,7 +799,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -856,16 +812,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -875,12 +823,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -888,16 +836,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -907,12 +847,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -920,16 +860,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -939,7 +871,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -952,16 +884,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
@@ -971,7 +895,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Juan Camilo Melchor Agudelo</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -984,16 +908,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
@@ -1003,12 +919,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1021,11 +937,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1035,12 +947,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1053,11 +965,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -1067,12 +975,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1085,16 +993,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
@@ -1103,7 +1003,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Nicolás Aros</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1121,16 +1021,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
@@ -1139,12 +1031,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1157,16 +1049,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
@@ -1175,12 +1059,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1198,11 +1082,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
@@ -1211,12 +1091,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1234,11 +1114,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
@@ -1247,12 +1123,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1270,16 +1146,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
@@ -1287,12 +1155,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1310,16 +1178,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
@@ -1327,7 +1187,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1350,16 +1210,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
@@ -1367,12 +1219,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1390,16 +1242,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -1407,12 +1251,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1430,28 +1274,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1479,28 +1311,20 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1523,28 +1347,20 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1567,23 +1383,15 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1611,27 +1419,15 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1664,22 +1460,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1712,27 +1500,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Federico Caruso Pérez</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1760,27 +1540,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1808,27 +1580,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1861,17 +1625,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1899,27 +1659,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1957,22 +1713,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2015,7 +1767,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2063,12 +1815,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2106,21 +1858,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Patricia Proniewska</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2158,16 +1906,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2210,16 +1954,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2262,21 +2002,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2314,21 +2050,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2351,11 +2083,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2375,12 +2103,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Andrey Ismagilov</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2418,21 +2146,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2470,21 +2194,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>Ana Claudia da Costa Dionisio Souza</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2531,7 +2251,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2583,7 +2303,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2635,7 +2355,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2679,6 +2399,318 @@
         </is>
       </c>
       <c r="J59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>M Isabel Villar</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Vanessa Bujaldon Pellicer</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Rossemary Castellanos</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Ramiro Aguilar Andrade</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Armando Aguilar Campos</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Ignacio Soldevilla</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-03-24 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -531,12 +531,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -551,12 +551,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -571,7 +571,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -591,12 +591,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -631,12 +631,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Raúl Martínez</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -651,12 +651,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raúl Martínez</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -671,7 +671,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -691,7 +691,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -711,12 +711,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Mohammad Gholinezhad</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -731,12 +731,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mohammad Gholinezhad</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -751,12 +751,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -775,7 +775,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -799,12 +799,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -823,12 +823,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -847,12 +847,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Juan Camilo Melchor Agudelo</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -871,7 +871,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -884,7 +884,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
@@ -895,7 +899,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Juan Camilo Melchor Agudelo</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -908,7 +912,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -947,12 +955,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -975,12 +983,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1003,12 +1011,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1031,12 +1039,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1049,7 +1057,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -1059,7 +1071,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1091,7 +1103,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1123,7 +1135,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1155,12 +1167,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1187,7 +1199,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1219,7 +1231,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1251,12 +1263,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1283,12 +1295,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1319,12 +1331,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1355,7 +1367,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1391,12 +1403,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1419,7 +1431,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -1427,12 +1443,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1467,7 +1483,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1507,12 +1523,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1547,7 +1563,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1580,7 +1596,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
     </row>
@@ -1675,7 +1695,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1719,12 +1739,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1767,12 +1787,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1863,12 +1883,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1911,12 +1931,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1959,12 +1979,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2007,12 +2027,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2055,12 +2075,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2083,7 +2103,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2094,11 +2118,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2151,12 +2171,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2179,11 +2199,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2194,7 +2210,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2251,7 +2271,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Gabriela La Cruz</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2303,7 +2323,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Margarita Cantero Guerrero</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2355,12 +2375,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Armando Aguilar Campos</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2407,12 +2427,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Ignacio Soldevilla</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2511,7 +2531,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Margarita Cantero Guerrero</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2615,7 +2635,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2667,7 +2687,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-03-25 16:11
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,12 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -491,12 +491,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -511,12 +511,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -531,12 +531,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -551,12 +551,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Mohammad Gholinezhad</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -591,12 +591,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -611,7 +611,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -631,12 +631,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Raúl Martínez</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -651,15 +651,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -671,7 +675,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -679,7 +683,11 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -691,7 +699,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -699,7 +707,11 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
@@ -711,7 +723,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mohammad Gholinezhad</t>
+          <t>Raúl Martínez</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -719,7 +731,11 @@
           <t>Joan</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -731,15 +747,19 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
@@ -751,12 +771,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -775,7 +795,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -799,12 +819,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Juan Camilo Melchor Agudelo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -823,12 +843,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -847,7 +867,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Juan Camilo Melchor Agudelo</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -860,7 +880,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
@@ -871,7 +895,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -899,7 +923,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -927,12 +951,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -955,12 +979,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -983,7 +1007,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1039,7 +1063,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1071,12 +1095,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1103,7 +1127,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1135,7 +1159,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1167,7 +1191,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1199,7 +1223,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1231,12 +1255,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1295,7 +1319,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1331,12 +1355,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1367,12 +1391,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1403,7 +1427,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1443,12 +1467,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1483,12 +1507,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1523,12 +1547,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1563,7 +1587,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1607,12 +1631,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1651,12 +1675,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1695,7 +1719,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1739,12 +1763,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1787,12 +1811,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1883,7 +1907,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1931,7 +1955,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Emilio Tornos Iniesta</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1959,11 +1983,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1974,17 +1994,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2027,12 +2051,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2075,7 +2099,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2118,17 +2142,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2166,12 +2194,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2199,7 +2231,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2219,12 +2255,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Ana Claudia da Costa Dionisio Souza</t>
+          <t>Gabriela La Cruz</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2271,7 +2307,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2323,7 +2359,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2375,12 +2411,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Armando Aguilar Campos</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2427,12 +2463,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Ignacio Soldevilla</t>
+          <t>Emilio Tornos Iniesta</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2479,12 +2515,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2523,214 +2559,6 @@
         </is>
       </c>
       <c r="J61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Margarita Cantero Guerrero</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Ramiro Aguilar Andrade</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Gabriela La Cruz</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P 2026-04-09 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M64"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mohammad Gholinezhad</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,7 +624,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -670,7 +670,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,12 +693,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -716,15 +716,19 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
@@ -739,12 +743,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -766,7 +770,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Juan Camilo Melchor Agudelo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -793,7 +797,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -820,7 +824,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -847,12 +851,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -874,12 +878,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -901,12 +905,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -928,12 +932,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Juan Camilo Melchor Agudelo</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -982,12 +986,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1009,7 +1013,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1022,7 +1026,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
@@ -1036,7 +1044,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1049,7 +1057,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
@@ -1063,12 +1075,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1094,12 +1106,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1125,12 +1137,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1156,7 +1168,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1187,12 +1199,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1205,7 +1217,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -1218,12 +1234,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1253,7 +1269,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1288,7 +1304,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1323,7 +1339,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1358,7 +1374,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1393,7 +1409,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1428,12 +1444,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1457,13 +1473,17 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1502,7 +1522,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1541,7 +1561,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1575,7 +1595,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1606,7 +1630,11 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
@@ -1619,12 +1647,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1705,12 +1733,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1748,12 +1776,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1834,12 +1862,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1860,7 +1888,11 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
@@ -1877,12 +1909,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1971,12 +2003,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2002,7 +2034,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
@@ -2018,12 +2054,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2069,12 +2105,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2105,27 +2141,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2171,12 +2207,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2222,12 +2258,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2258,17 +2294,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2324,12 +2360,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2375,7 +2411,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Ramiro Aguilar Andrade</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2411,7 +2447,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2426,7 +2466,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2481,7 +2521,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2536,12 +2576,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2646,7 +2686,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2701,7 +2741,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2753,61 +2793,6 @@
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Alexei Levitchi</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P 2026-04-10 10:45
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1075,12 +1075,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1106,12 +1106,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1234,7 +1234,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1304,7 +1304,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1339,7 +1339,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1409,7 +1409,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1438,13 +1438,17 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1522,7 +1526,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1647,12 +1651,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1690,12 +1694,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1776,12 +1780,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1819,7 +1823,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1862,12 +1866,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1956,7 +1960,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1987,7 +1991,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
@@ -2003,12 +2011,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2054,12 +2062,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2105,7 +2113,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2141,27 +2149,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2192,27 +2200,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2258,7 +2266,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2294,7 +2302,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2309,12 +2321,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Damian Vallejos</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2345,7 +2357,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2360,12 +2376,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2396,7 +2412,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2411,12 +2431,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ramiro Aguilar Andrade</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2466,12 +2486,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2521,7 +2541,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2576,12 +2596,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2631,12 +2651,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2686,7 +2706,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2738,61 +2758,6 @@
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Rossemary Castellanos</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P 2026-04-14 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M62"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -670,7 +670,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,12 +693,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -716,12 +716,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -743,7 +743,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -770,7 +770,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Juan Camilo Melchor Agudelo</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -824,7 +824,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -851,12 +851,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -878,7 +878,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Juan Camilo Melchor Agudelo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -905,12 +905,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -932,12 +932,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -986,12 +986,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -999,7 +999,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -1013,12 +1017,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1026,12 +1030,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1044,7 +1048,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1075,12 +1079,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1106,12 +1110,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1137,12 +1141,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1168,12 +1172,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1186,7 +1190,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -1234,7 +1242,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1269,7 +1277,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1339,7 +1347,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1374,7 +1382,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1409,12 +1417,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1448,12 +1456,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1487,7 +1495,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1526,12 +1534,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1560,17 +1568,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1591,7 +1603,11 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
@@ -1599,21 +1615,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1634,11 +1646,7 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
@@ -1646,7 +1654,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1737,12 +1749,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1780,12 +1792,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1806,7 +1818,11 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
@@ -1823,7 +1839,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1849,7 +1865,11 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
@@ -1960,12 +1980,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2011,7 +2031,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2062,12 +2082,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2098,22 +2118,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2164,12 +2184,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2200,27 +2220,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2321,7 +2341,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Damian Vallejos</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2376,7 +2396,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2431,7 +2451,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>M Isabel Villar</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2486,7 +2506,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2541,7 +2561,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2596,12 +2616,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Mariia Zaitseva</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2651,12 +2671,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Mariia Zaitseva</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2703,61 +2723,6 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Rossemary Castellanos</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P 2026-04-14 09:25
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,7 +532,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,7 +647,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -670,12 +670,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -693,15 +693,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
@@ -716,12 +720,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Juan Camilo Melchor Agudelo</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -878,12 +882,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Juan Camilo Melchor Agudelo</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -959,7 +963,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -986,12 +990,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -999,11 +1003,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -1110,12 +1110,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1141,12 +1141,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1172,12 +1172,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1190,11 +1190,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -1277,7 +1273,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1382,12 +1378,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1417,12 +1413,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1446,22 +1442,18 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1495,12 +1487,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1534,12 +1526,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1568,11 +1560,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1620,7 +1608,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1663,12 +1651,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1749,12 +1737,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1792,7 +1780,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1818,11 +1806,7 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
@@ -1839,12 +1823,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1886,12 +1870,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1933,7 +1917,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1980,12 +1964,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2011,11 +1995,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
@@ -2031,7 +2011,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2082,7 +2062,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2118,22 +2098,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2286,12 +2266,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2332,21 +2312,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2396,12 +2372,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2451,12 +2427,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>M Isabel Villar</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2506,12 +2482,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2561,12 +2537,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2616,12 +2592,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-04-15 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,7 +555,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -670,12 +670,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -882,12 +882,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -909,12 +909,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -936,12 +936,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -949,7 +949,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
@@ -963,7 +967,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -977,7 +981,11 @@
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
@@ -990,7 +998,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1004,7 +1012,11 @@
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
@@ -1017,7 +1029,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1030,12 +1042,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1048,12 +1060,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1079,7 +1091,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1141,12 +1153,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1172,12 +1184,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1308,7 +1320,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1343,7 +1355,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1378,12 +1390,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1413,12 +1425,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1448,12 +1460,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1487,12 +1499,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1737,12 +1749,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1780,12 +1792,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1806,7 +1818,11 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
@@ -1823,7 +1839,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1870,12 +1886,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1917,12 +1933,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1948,7 +1964,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
@@ -1964,12 +1984,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1995,28 +2015,32 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2062,12 +2086,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2113,12 +2137,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2164,7 +2188,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2215,12 +2239,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Alexei Levitchi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2251,7 +2275,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2266,7 +2294,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2312,12 +2340,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2372,12 +2404,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2592,12 +2624,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P 2026-04-20 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:M59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,18 +624,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -647,15 +651,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -670,7 +678,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Juan Camilo Melchor Agudelo</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -678,7 +686,11 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
@@ -693,12 +705,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -720,7 +732,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Juan Camilo Melchor Agudelo</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -747,7 +759,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -774,7 +786,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -801,7 +813,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -828,22 +840,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -855,12 +867,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -868,7 +880,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
@@ -882,12 +898,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -895,7 +911,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
@@ -909,12 +929,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -922,7 +942,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
@@ -936,7 +960,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -967,12 +991,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -980,12 +1004,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
@@ -998,7 +1022,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1091,12 +1115,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1109,7 +1133,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -1122,7 +1150,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1140,7 +1168,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -1153,12 +1185,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1171,7 +1203,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -1184,12 +1220,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1202,7 +1238,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -1215,12 +1255,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1250,7 +1290,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1285,12 +1325,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1355,12 +1395,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1390,7 +1430,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1460,12 +1500,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1538,12 +1578,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1577,12 +1617,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1603,11 +1643,7 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
@@ -1615,7 +1651,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1663,12 +1703,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1749,12 +1789,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1775,7 +1815,11 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
@@ -1783,11 +1827,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1933,12 +1973,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1984,12 +2024,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2020,22 +2060,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2086,12 +2126,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2122,17 +2162,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2188,12 +2228,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2224,7 +2264,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2239,7 +2283,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Alexei Levitchi</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2294,7 +2338,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2404,7 +2448,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2514,12 +2558,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2569,7 +2613,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2621,116 +2665,6 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Ricardo Gabriel Castro abad</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Mariia Zaitseva</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-04-20 18:51
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M59"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -578,7 +578,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -624,22 +624,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -651,22 +647,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -678,12 +674,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Juan Camilo Melchor Agudelo</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -705,7 +701,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Juan Camilo Melchor Agudelo</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -732,7 +728,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -759,7 +755,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -786,7 +782,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -813,7 +809,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -840,22 +836,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -1022,27 +1018,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1053,7 +1049,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1066,12 +1062,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1084,7 +1080,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1115,12 +1111,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1133,11 +1129,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -1150,12 +1142,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1185,12 +1177,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1220,7 +1212,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1255,12 +1247,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1290,12 +1282,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1325,12 +1317,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1360,7 +1352,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1395,12 +1387,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1430,12 +1422,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1465,12 +1457,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1500,12 +1492,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1529,22 +1521,18 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1578,12 +1566,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1617,12 +1605,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1651,21 +1639,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1703,12 +1687,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1729,7 +1713,11 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
@@ -1737,16 +1725,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1789,12 +1773,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1815,11 +1799,7 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
@@ -1827,17 +1807,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1858,11 +1842,7 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
@@ -1879,12 +1859,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1973,12 +1953,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2004,11 +1984,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
@@ -2075,7 +2051,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2126,12 +2102,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2162,27 +2138,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2213,22 +2189,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2264,11 +2240,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2283,12 +2255,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Vanessa Mercedes Plaza Aguilar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2338,7 +2310,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2393,7 +2365,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2448,12 +2420,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2503,12 +2475,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2558,12 +2530,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2613,12 +2585,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Vanessa Mercedes Plaza Aguilar</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2665,6 +2637,61 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Vanessa Bujaldon Pellicer</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-04-27 09:25
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,7 +555,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Alejandro Sebastià</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -578,18 +578,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -601,7 +605,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -964,27 +968,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1030,12 +1038,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1065,7 +1073,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1100,7 +1108,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1135,7 +1143,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1170,12 +1178,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1240,12 +1248,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1310,12 +1318,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1345,32 +1353,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
@@ -1380,12 +1388,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1415,7 +1423,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1485,12 +1493,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1520,7 +1528,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1594,12 +1602,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1637,12 +1645,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1680,7 +1688,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1723,7 +1731,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1766,7 +1774,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1809,7 +1817,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1895,12 +1903,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1942,7 +1950,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1989,12 +1997,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2036,12 +2044,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2072,27 +2080,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2123,17 +2131,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2189,12 +2197,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Vanesa Perez Ramirez</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2240,12 +2248,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2276,7 +2284,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2291,7 +2303,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2346,7 +2358,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Francesco Eirado Enes</t>
+          <t>Minu Campoy</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2401,12 +2413,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Minu Campoy</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2456,12 +2468,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Ana Cristina Urdaneta Flores</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2511,7 +2523,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Rossemary Castellanos</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2566,12 +2578,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ana Cristina Urdaneta Flores</t>
+          <t>Francesco Eirado Enes</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2621,12 +2633,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Rossemary Castellanos</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-04-29 09:25
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M59"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -520,7 +520,11 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -532,18 +536,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -555,18 +563,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alejandro Sebastià</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -578,12 +590,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -605,12 +617,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -648,7 +660,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -659,22 +675,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -686,12 +706,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -699,7 +719,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -713,7 +737,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -726,7 +750,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -740,7 +768,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -753,7 +781,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -761,7 +793,11 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -780,8 +816,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -807,8 +851,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -821,12 +873,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -834,8 +886,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -848,12 +908,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Juan Camilo Melchor Agudelo</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -861,8 +921,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -875,12 +943,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -893,7 +961,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -906,12 +978,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -924,7 +996,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -937,12 +1013,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -955,7 +1031,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -968,7 +1048,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1003,7 +1083,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1038,12 +1118,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1073,7 +1153,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1108,32 +1188,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
@@ -1143,12 +1223,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1178,12 +1258,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1213,12 +1293,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1248,12 +1328,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1283,7 +1363,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1312,18 +1392,22 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1347,53 +1431,61 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1417,18 +1509,26 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1452,18 +1552,26 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1487,18 +1595,26 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1522,18 +1638,26 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1557,13 +1681,21 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1597,17 +1729,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1645,7 +1781,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1688,12 +1824,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1714,7 +1850,11 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
@@ -1731,12 +1871,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1757,24 +1897,28 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1800,8 +1944,16 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
@@ -1817,12 +1969,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1843,24 +1995,32 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1891,24 +2051,32 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1934,8 +2102,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1981,8 +2157,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1997,7 +2181,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2028,8 +2212,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2044,7 +2236,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2080,7 +2272,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2095,12 +2291,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2141,17 +2337,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2182,7 +2382,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2197,7 +2401,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Vanesa Perez Ramirez</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2233,453 +2437,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Dioulde Diao Gano</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Ricardo Gabriel Castro abad</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Minu Campoy</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Sabina Planas Bonell</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Ana Cristina Urdaneta Flores</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Vanessa Bujaldon Pellicer</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Francesco Eirado Enes</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Rossemary Castellanos</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-04-30 09:58
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -1293,7 +1293,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1328,12 +1328,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1357,18 +1357,22 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-04 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:M56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,22 +509,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -536,22 +532,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -563,22 +555,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Renata Khazieva</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -590,22 +578,18 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -617,22 +601,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -644,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -660,11 +640,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -675,7 +651,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -683,18 +659,14 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -706,26 +678,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -737,7 +705,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -745,18 +713,14 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -768,66 +732,58 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -838,7 +794,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -856,11 +812,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -873,12 +825,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -886,11 +838,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>✅</t>
@@ -908,12 +856,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -926,11 +874,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -943,12 +887,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -961,29 +905,29 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1013,12 +957,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1048,7 +992,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1083,7 +1027,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1118,12 +1062,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1153,7 +1097,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1188,32 +1132,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
@@ -1223,12 +1167,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1258,12 +1202,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1293,12 +1237,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1328,12 +1272,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1357,56 +1301,48 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1435,22 +1371,18 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1474,22 +1406,18 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1513,26 +1441,18 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1561,21 +1481,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1604,21 +1520,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1647,21 +1559,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1690,16 +1598,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1742,12 +1646,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1785,12 +1689,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1828,12 +1732,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1854,11 +1758,7 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
@@ -1875,12 +1775,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1901,33 +1801,29 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1948,16 +1844,8 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
@@ -1973,12 +1861,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1999,37 +1887,29 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2050,16 +1930,8 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
@@ -2075,12 +1947,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2106,16 +1978,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2130,12 +1994,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2166,31 +2030,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2221,11 +2077,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2240,12 +2092,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2286,21 +2138,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2331,11 +2179,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2350,12 +2194,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2405,12 +2249,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2457,6 +2301,281 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Ricardo Gabriel Castro abad</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sabina Planas Bonell</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ROCIO ANA ARIAS</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Marine Fernandez</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Vanessa Bujaldon Pellicer</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-05 09:41
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M56"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,15 +469,20 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>Dates_1</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Python 3</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>PBI 1</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>PBI 2</t>
         </is>
@@ -505,16 +510,17 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -528,16 +534,17 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Renata Khazieva</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -551,16 +558,17 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Renata Khazieva</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -574,16 +582,17 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -597,16 +606,17 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -620,26 +630,23 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -647,11 +654,12 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -662,11 +670,7 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -674,26 +678,23 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -701,26 +702,23 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -728,90 +726,69 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
@@ -821,29 +798,22 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -852,30 +822,27 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -883,11 +850,12 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -895,57 +863,42 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -953,34 +906,27 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
@@ -988,86 +934,81 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1075,11 +1016,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1093,16 +1030,17 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1115,11 +1053,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1128,16 +1062,17 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1150,11 +1085,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -1163,6 +1094,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1198,11 +1130,12 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1233,16 +1166,17 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1268,11 +1202,12 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1303,51 +1238,53 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1373,16 +1310,17 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1408,16 +1346,17 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1430,11 +1369,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -1442,17 +1377,22 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1476,17 +1416,14 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1515,22 +1452,19 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1554,22 +1488,19 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1593,65 +1524,55 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1675,26 +1596,19 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1718,26 +1632,19 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1761,21 +1668,18 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
+      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1804,26 +1708,23 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1847,26 +1748,23 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
+      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1890,26 +1788,23 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
+      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1933,21 +1828,18 @@
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1973,19 +1865,16 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -1994,12 +1883,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2020,28 +1909,25 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2067,23 +1953,16 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2092,12 +1971,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2118,37 +1997,30 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2169,23 +2041,16 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2194,12 +2059,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2220,27 +2085,16 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2249,12 +2103,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2275,27 +2129,16 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2304,7 +2147,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2340,31 +2183,24 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
+      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2390,22 +2226,15 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2414,7 +2243,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2445,22 +2274,15 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2469,12 +2291,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2505,17 +2327,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2524,7 +2343,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2560,17 +2379,458 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Tatiana Lukina</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Sabina Planas Bonell</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Ricardo Gabriel Castro abad</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Marine Fernandez</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Dioulde Diao Gano</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ROCIO ANA ARIAS</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Noelia Solano Romero</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Vanessa Bujaldon Pellicer</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-06 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -515,12 +515,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Renata Khazieva</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -563,12 +563,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -587,12 +587,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -635,12 +635,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -659,12 +659,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Renata Khazieva</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -683,12 +683,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -707,12 +707,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -731,12 +731,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -779,12 +779,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -803,18 +803,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -827,12 +831,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -855,12 +859,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -939,7 +943,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -971,27 +975,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1067,27 +1071,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1099,12 +1103,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1117,11 +1121,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -1129,18 +1129,22 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1171,12 +1175,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1207,7 +1211,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1243,7 +1247,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1279,12 +1283,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1315,12 +1319,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1351,12 +1355,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1369,7 +1373,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -1377,11 +1385,7 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1495,32 +1499,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
@@ -1531,32 +1535,32 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
@@ -1567,7 +1571,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1603,12 +1607,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1633,18 +1637,22 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1679,7 +1687,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1719,12 +1727,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1759,7 +1767,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1799,12 +1807,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1834,12 +1842,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1927,12 +1939,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1971,12 +1983,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2015,12 +2027,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2059,12 +2071,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2103,12 +2115,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2147,12 +2159,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2178,11 +2190,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
@@ -2190,12 +2198,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2243,12 +2255,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2274,7 +2286,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
@@ -2291,7 +2307,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2328,27 +2344,27 @@
         </is>
       </c>
       <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M55" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2380,22 +2396,22 @@
         </is>
       </c>
       <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M56" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2432,27 +2448,27 @@
         </is>
       </c>
       <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2559,12 +2575,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2615,12 +2631,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2783,12 +2799,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-07 09:25
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -491,7 +491,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -903,7 +903,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -931,7 +935,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -943,27 +951,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -975,7 +983,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1007,12 +1015,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1020,12 +1028,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
@@ -1039,12 +1047,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1057,7 +1065,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1071,27 +1083,31 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1103,12 +1119,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1121,7 +1137,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -1129,22 +1149,18 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1175,12 +1191,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1211,12 +1227,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1247,12 +1263,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1283,12 +1299,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1301,11 +1317,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
@@ -1313,18 +1325,22 @@
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1355,7 +1371,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1391,12 +1407,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1427,32 +1443,32 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
@@ -1463,32 +1479,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
@@ -1499,7 +1515,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1571,12 +1587,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1601,18 +1617,22 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1647,7 +1667,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1687,12 +1707,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1727,12 +1747,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1807,12 +1827,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1851,12 +1871,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1895,12 +1915,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1983,12 +2003,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2071,12 +2091,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2115,12 +2135,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2411,7 +2431,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2448,7 +2468,11 @@
         </is>
       </c>
       <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M57" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2463,7 +2487,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2519,12 +2543,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2575,7 +2599,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2631,12 +2655,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2687,12 +2711,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2743,12 +2767,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-07 11:12
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N64"/>
+  <dimension ref="A1:M76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,31 +469,22 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Dates_1</t>
+          <t>Python 3</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Python 3</t>
+          <t>PBI 1</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>PBI 1</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
           <t>PBI 2</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Juan Claros</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -510,17 +501,12 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Francisco José Jiménez Fernández</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -534,17 +520,12 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Alicia Domínguez</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -558,17 +539,12 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Hugo Nascimento</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -582,17 +558,12 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Silvia Vilches</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -606,17 +577,12 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Pau Serrano</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -630,17 +596,12 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Jorge Kundig</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -654,17 +615,16 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Renata Khazieva</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -678,17 +638,16 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -702,12 +661,11 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -726,12 +684,11 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -750,12 +707,11 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -774,14 +730,9 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Violeta Correa</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -798,27 +749,18 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Arnau Rosich Giménez</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -826,27 +768,18 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Biel Domènech</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -854,12 +787,11 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -870,11 +802,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -882,94 +810,67 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Renata Khazieva</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -978,29 +879,20 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
@@ -1010,29 +902,20 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -1042,34 +925,21 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -1078,34 +948,21 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -1114,34 +971,17 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Hector Morales</t>
-        </is>
-      </c>
+      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -1150,34 +990,17 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Christopher Rancel</t>
-        </is>
-      </c>
+      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -1186,35 +1009,26 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
@@ -1222,35 +1036,26 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
@@ -1258,35 +1063,26 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
@@ -1294,89 +1090,78 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1384,11 +1169,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1402,17 +1183,16 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1425,11 +1205,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
@@ -1438,125 +1214,117 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1582,12 +1350,11 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1617,22 +1384,17 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1657,22 +1419,17 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1697,22 +1454,17 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1737,22 +1489,17 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1765,29 +1512,24 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1817,22 +1559,17 @@
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1857,21 +1594,12 @@
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1901,153 +1629,117 @@
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2077,26 +1769,17 @@
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2120,27 +1803,22 @@
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2164,27 +1842,22 @@
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2205,34 +1878,25 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2253,29 +1917,20 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2301,38 +1956,25 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2353,38 +1995,25 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2405,16 +2034,8 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
@@ -2426,17 +2047,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2457,16 +2077,8 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
@@ -2478,21 +2090,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2513,16 +2120,8 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
@@ -2534,21 +2133,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ROCIO ANA ARIAS</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2569,16 +2163,8 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
@@ -2590,16 +2176,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2625,16 +2206,8 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
@@ -2646,21 +2219,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2681,16 +2249,8 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
@@ -2702,21 +2262,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2737,16 +2292,8 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
@@ -2758,21 +2305,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2793,16 +2335,8 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
@@ -2814,16 +2348,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2854,11 +2383,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
@@ -2870,7 +2395,642 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr">
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Santiago Alvarez Salvado</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Elisa Volk</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Federico Urbina</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Tatiana Lukina</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Ricardo Gabriel Castro abad</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Marine Fernandez</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Dioulde Diao Gano</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Giorgia Calvagna</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ROCIO ANA ARIAS</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Sabina Planas Bonell</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Noelia Solano Romero</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Vanessa Bujaldon Pellicer</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-07 11:15
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M76"/>
+  <dimension ref="A1:M64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,7 +484,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Juan Claros</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -503,10 +507,14 @@
       <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Francisco José Jiménez Fernández</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -522,10 +530,14 @@
       <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Alicia Domínguez</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -541,10 +553,14 @@
       <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hugo Nascimento</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -560,10 +576,14 @@
       <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Silvia Vilches</t>
+        </is>
+      </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -579,10 +599,14 @@
       <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pau Serrano</t>
+        </is>
+      </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -598,10 +622,14 @@
       <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jorge Kundig</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -619,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Renata Khazieva</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -642,12 +670,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -665,7 +693,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -688,7 +716,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -711,7 +739,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -732,7 +760,11 @@
       <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Violeta Correa</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -751,16 +783,24 @@
       <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Arnau Rosich Giménez</t>
+        </is>
+      </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -770,16 +810,24 @@
       <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Biel Domènech</t>
+        </is>
+      </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -791,7 +839,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -802,7 +850,11 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -814,19 +866,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Renata Khazieva</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -837,19 +897,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -860,17 +928,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -883,16 +959,24 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
@@ -906,16 +990,24 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -929,17 +1021,29 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -952,17 +1056,29 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -973,15 +1089,31 @@
       <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Hector Morales</t>
+        </is>
+      </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -992,15 +1124,31 @@
       <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Christopher Rancel</t>
+        </is>
+      </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -1013,22 +1161,30 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
@@ -1040,22 +1196,30 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
@@ -1067,22 +1231,30 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
@@ -1094,58 +1266,66 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
@@ -1156,12 +1336,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1169,7 +1349,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1187,12 +1371,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1205,7 +1389,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
@@ -1218,28 +1406,32 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
@@ -1249,32 +1441,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
@@ -1284,32 +1476,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
@@ -1319,12 +1511,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1354,7 +1546,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1383,18 +1575,22 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1418,18 +1614,22 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1453,18 +1653,22 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1488,18 +1692,22 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1512,7 +1720,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
@@ -1529,7 +1741,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1558,18 +1770,22 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1593,13 +1809,21 @@
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Vanina Tonzo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1628,118 +1852,150 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Erik Subirats</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1768,18 +2024,26 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1808,17 +2072,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1847,17 +2115,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1878,7 +2150,11 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
@@ -1886,17 +2162,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1917,7 +2197,11 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
@@ -1925,12 +2209,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1956,25 +2244,37 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1995,9 +2295,21 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2008,12 +2320,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2034,29 +2346,37 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Dioulde Diao Gano</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2077,9 +2397,21 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2094,12 +2426,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Erik Subirats</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2120,9 +2452,21 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2137,12 +2481,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>ROCIO ANA ARIAS</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2163,9 +2507,21 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2180,7 +2536,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Sabina Planas Bonell</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2206,9 +2562,21 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L60" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2223,12 +2591,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2249,9 +2617,21 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2266,12 +2646,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2292,9 +2672,21 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L62" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2309,12 +2701,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2335,9 +2727,21 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2352,7 +2756,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2383,654 +2787,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Santiago Alvarez Salvado</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Elisa Volk</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Federico Urbina</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Tatiana Lukina</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Ricardo Gabriel Castro abad</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Marine Fernandez</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Dioulde Diao Gano</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Giorgia Calvagna</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>ROCIO ANA ARIAS</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Sabina Planas Bonell</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Noelia Solano Romero</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Vanessa Bujaldon Pellicer</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-18 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:M64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Renata Khazieva</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Renata Khazieva</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -670,7 +670,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,7 +693,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -716,7 +716,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -739,7 +739,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -789,12 +789,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -816,12 +816,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -843,12 +843,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -870,12 +870,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -886,11 +886,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -901,12 +897,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -917,11 +913,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -932,26 +924,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
@@ -963,26 +951,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
@@ -994,26 +978,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
@@ -1025,31 +1005,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1060,31 +1036,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1095,12 +1067,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1108,11 +1080,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1130,12 +1098,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1148,11 +1116,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -1165,7 +1129,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1183,11 +1147,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -1235,12 +1195,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1270,7 +1230,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1305,32 +1265,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
@@ -1340,12 +1300,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1375,32 +1335,32 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
@@ -1445,32 +1405,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
@@ -1480,85 +1440,77 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1587,11 +1539,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1636,12 +1584,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1675,40 +1623,40 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
@@ -1753,7 +1701,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1787,21 +1735,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1830,21 +1774,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1873,16 +1813,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1916,21 +1852,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1968,7 +1900,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1994,11 +1926,7 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
@@ -2015,7 +1943,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2041,11 +1969,7 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
@@ -2062,7 +1986,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2088,11 +2012,7 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
@@ -2109,7 +2029,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Vanina Tonzo</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2135,11 +2055,7 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
@@ -2156,12 +2072,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2187,32 +2103,28 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2238,27 +2150,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Federico Urbina</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2284,17 +2192,13 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2309,12 +2213,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2340,16 +2244,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2364,7 +2260,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Dioulde Diao Gano</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2410,16 +2306,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2465,21 +2357,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Noelia Solano Romero</t>
+          <t>Federico Urbina</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2529,12 +2417,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2584,12 +2472,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Noelia Solano Romero</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2639,7 +2527,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Sabina Planas Bonell</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2691,6 +2579,171 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Marine Fernandez</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Sabina Planas Bonell</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Ricardo Gabriel Castro abad</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-19 09:30
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M64"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Renata Khazieva</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -670,12 +670,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -693,12 +693,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -716,12 +716,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -739,12 +739,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -762,7 +762,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -773,11 +773,7 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -789,22 +785,18 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -816,22 +808,18 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -843,22 +831,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -870,7 +854,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -881,11 +865,7 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -924,7 +904,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -951,12 +931,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -978,7 +958,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1005,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1021,11 +1001,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1036,12 +1012,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1052,11 +1028,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1067,27 +1039,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -1098,27 +1070,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -1129,27 +1101,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1160,67 +1132,63 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
@@ -1230,32 +1198,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
@@ -1265,12 +1233,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1278,11 +1246,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1294,18 +1258,22 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1335,12 +1303,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1405,12 +1373,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1440,82 +1408,90 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1539,52 +1515,56 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1623,46 +1603,46 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1691,17 +1671,17 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1735,12 +1715,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1774,17 +1758,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1813,17 +1801,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1852,17 +1844,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1883,7 +1879,11 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
@@ -1900,7 +1900,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1928,7 +1928,11 @@
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1943,12 +1947,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1969,29 +1973,37 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2012,9 +2024,21 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2029,12 +2053,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2055,9 +2079,21 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2072,12 +2108,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2103,8 +2139,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2119,12 +2163,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2150,595 +2194,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Florencia Di Stefano</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Jordi Lamarca</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Elisa Volk</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Tatiana Lukina</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Federico Urbina</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Giorgia Calvagna</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Noelia Solano Romero</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Vanessa Bujaldon Pellicer</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Marine Fernandez</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Sabina Planas Bonell</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Ricardo Gabriel Castro abad</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-21 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -532,7 +532,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,7 +647,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -670,7 +670,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,12 +693,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -716,12 +716,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -739,12 +739,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -762,18 +762,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -785,18 +789,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -808,18 +816,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -831,18 +843,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -854,7 +870,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -865,7 +881,11 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -877,12 +897,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -904,12 +924,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -931,12 +951,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -958,12 +978,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -985,7 +1005,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1101,12 +1121,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1122,7 +1142,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
@@ -1132,12 +1156,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1153,7 +1177,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
@@ -1163,12 +1191,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1198,12 +1226,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1268,12 +1296,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1303,12 +1331,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1338,12 +1366,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1373,12 +1401,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1402,52 +1430,56 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1486,7 +1518,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1525,51 +1557,51 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1603,7 +1635,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1632,22 +1664,22 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1671,7 +1703,11 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M42" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1681,7 +1717,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1724,7 +1760,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1767,12 +1803,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2108,12 +2144,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2163,12 +2199,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-21 14:16
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -624,7 +624,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -670,7 +670,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,12 +693,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -716,12 +716,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -739,18 +739,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
@@ -762,12 +766,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -789,12 +793,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -816,12 +820,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -843,12 +847,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -870,12 +874,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -897,7 +901,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -924,7 +928,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -951,7 +955,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -978,12 +982,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1005,12 +1009,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1032,7 +1036,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1048,7 +1052,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1296,12 +1304,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1331,12 +1339,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1360,39 +1368,47 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -1401,7 +1417,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1440,46 +1456,46 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1518,12 +1534,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1557,12 +1573,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1661,7 +1677,11 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-26 09:31
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,7 +624,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -670,7 +670,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,7 +693,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -716,12 +716,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -766,12 +766,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -793,12 +793,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -820,12 +820,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -847,12 +847,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -874,7 +874,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -928,7 +928,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -955,12 +955,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -982,12 +982,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1009,7 +1009,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1025,7 +1025,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1036,12 +1040,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1067,12 +1071,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1269,12 +1273,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1282,7 +1286,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1294,17 +1302,13 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1333,85 +1337,89 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1651,12 +1659,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1677,14 +1685,14 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M41" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1694,7 +1702,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1737,7 +1745,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1780,12 +1788,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1823,7 +1831,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1866,12 +1874,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1892,7 +1900,11 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
@@ -1909,7 +1921,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1935,13 +1947,13 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1956,12 +1968,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1982,8 +1994,16 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K48" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1994,16 +2014,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2039,22 +2055,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2109,7 +2125,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2164,12 +2180,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2219,12 +2235,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-27 09:24
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,7 +647,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -670,7 +670,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,7 +693,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -716,7 +716,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -739,22 +739,18 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
@@ -766,22 +762,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -793,7 +785,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -804,11 +796,7 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -820,7 +808,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -831,11 +819,7 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -847,22 +831,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -874,7 +854,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -901,12 +881,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -928,7 +908,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -955,12 +935,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -982,12 +962,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1009,12 +989,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1025,11 +1005,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1040,12 +1016,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1071,12 +1047,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1102,7 +1078,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1133,12 +1109,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1154,11 +1130,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
@@ -1168,7 +1140,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1189,11 +1161,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
@@ -1203,12 +1171,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1224,11 +1192,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
@@ -1238,7 +1202,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1259,11 +1223,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
@@ -1273,32 +1233,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
@@ -1308,46 +1268,42 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1373,11 +1329,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
@@ -1386,85 +1338,77 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1493,61 +1437,57 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1581,7 +1521,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1620,12 +1560,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1659,12 +1599,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1693,16 +1633,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1736,16 +1672,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1779,16 +1711,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1831,12 +1759,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1874,7 +1802,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1900,11 +1828,7 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
@@ -1921,12 +1845,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1949,11 +1873,7 @@
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1968,12 +1888,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1994,32 +1914,24 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2045,16 +1957,8 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
@@ -2070,12 +1974,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2096,21 +2000,13 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2125,7 +2021,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2171,16 +2067,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2216,11 +2108,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2235,7 +2123,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2271,17 +2159,284 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Florencia Di Stefano</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Vanessa Bujaldon Pellicer</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Ricardo Gabriel Castro abad</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Giorgia Calvagna</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Elisa Volk</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-28 09:26
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -1303,7 +1303,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1338,7 +1338,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1373,32 +1373,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
@@ -1408,33 +1408,37 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
@@ -1443,7 +1447,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-28 10:13
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -1233,32 +1233,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
@@ -1268,7 +1268,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1303,12 +1303,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1373,32 +1373,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
@@ -1408,7 +1408,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1447,51 +1447,51 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1525,12 +1525,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1564,7 +1564,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1603,12 +1603,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1642,51 +1642,51 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1715,17 +1715,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1806,7 +1810,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1892,7 +1896,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2076,12 +2080,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2127,7 +2131,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Florencia Di Stefano</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2153,17 +2157,17 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2178,7 +2182,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2204,7 +2208,11 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J54" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2229,12 +2237,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Ricardo Gabriel Castro abad</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2284,7 +2292,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Giorgia Calvagna</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2339,7 +2347,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Elisa Volk</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2394,7 +2402,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-02 09:34
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M58"/>
+  <dimension ref="A1:M76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,7 +647,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -670,7 +670,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -693,12 +693,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -716,12 +716,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Sandra Valero Garcia</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -739,12 +739,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -762,7 +762,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -785,18 +785,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -808,18 +812,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -831,18 +839,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -854,12 +866,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -881,12 +893,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -897,7 +909,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -908,12 +924,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -924,7 +940,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -935,12 +955,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -951,7 +971,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -962,12 +986,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -978,7 +1002,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -989,12 +1017,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1005,7 +1033,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1016,27 +1048,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1047,12 +1079,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1078,12 +1110,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1099,7 +1131,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
@@ -1109,27 +1145,31 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1140,12 +1180,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1161,7 +1201,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
@@ -1171,7 +1215,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1192,7 +1236,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
@@ -1202,12 +1250,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1223,7 +1271,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
@@ -1233,32 +1285,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
@@ -1268,7 +1320,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1303,12 +1355,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1338,12 +1390,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1373,12 +1425,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1408,12 +1460,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1434,11 +1486,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
@@ -1447,90 +1495,86 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1564,12 +1608,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1642,46 +1686,46 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1715,21 +1759,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1758,21 +1798,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1785,11 +1821,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
@@ -1810,12 +1842,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1853,7 +1885,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1896,12 +1928,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1939,12 +1971,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1982,12 +2014,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2009,11 +2041,7 @@
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
@@ -2029,32 +2057,32 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2065,22 +2093,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2106,16 +2126,8 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
@@ -2131,7 +2143,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Florencia Di Stefano</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2158,16 +2170,8 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2182,7 +2186,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2208,21 +2212,9 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2237,12 +2229,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2263,21 +2255,9 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2292,12 +2272,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2323,16 +2303,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2347,12 +2319,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2378,16 +2350,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2402,7 +2366,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2433,22 +2397,968 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Roger Defez</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Tatiana Lukina</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Vanina Tonzo</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Santiago Alvarez Salvado</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Marcos Molina</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Hamza Messaoudi Basaid</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Dídac Petit</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Florencia Di Stefano</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Arnau Rosich Giménez</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Jordi Lamarca</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Elisa Volk</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Giorgia Calvagna</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Ricardo Gabriel Castro abad</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Vanessa Bujaldon Pellicer</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Marine Fernandez</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Jose Manuel Romero</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Timan (Nakta) samipour</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Raúl Martínez</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-04 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -878,7 +878,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -909,7 +909,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -971,27 +971,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1002,27 +1002,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1054,7 +1054,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
@@ -1064,12 +1068,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1204,12 +1208,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1239,7 +1243,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1449,32 +1453,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
@@ -1484,12 +1488,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1513,13 +1517,17 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1558,7 +1566,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1597,90 +1605,90 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1714,40 +1722,40 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-08 09:38
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,7 +532,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -555,7 +555,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -578,7 +578,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -624,18 +624,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -647,18 +651,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -670,7 +678,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -681,7 +689,11 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -693,7 +705,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -704,7 +716,11 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -716,12 +732,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -743,12 +759,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -770,12 +786,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -797,7 +813,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -824,7 +840,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -851,12 +867,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -878,7 +894,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -909,27 +925,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -940,12 +956,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -971,27 +987,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1002,12 +1018,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1023,7 +1039,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
@@ -1033,32 +1053,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
@@ -1068,7 +1088,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1103,12 +1123,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1138,12 +1158,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1173,12 +1193,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1208,12 +1228,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1383,12 +1403,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1418,7 +1438,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1453,32 +1473,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
@@ -1488,40 +1508,40 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1566,7 +1586,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1605,40 +1625,40 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1683,79 +1703,79 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1800,7 +1820,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1843,12 +1863,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1886,12 +1906,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1929,7 +1949,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1972,45 +1992,45 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2058,12 +2078,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2101,7 +2121,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2144,12 +2164,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2187,55 +2207,55 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>emmanuel Gonzalez Moreno</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2324,7 +2344,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2371,12 +2391,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>emmanuel Gonzalez Moreno</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2465,12 +2485,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2501,22 +2521,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2567,7 +2587,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2618,12 +2638,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2644,17 +2664,17 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L62" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2669,12 +2689,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2695,7 +2715,11 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2711,11 +2735,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2936,7 +2956,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Giorgia Calvagna</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3046,12 +3066,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3156,12 +3176,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3211,7 +3231,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Raúl Martínez</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3263,61 +3283,6 @@
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Raúl Martínez</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-10 09:23
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -1275,12 +1275,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1310,7 +1310,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1345,7 +1345,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1380,7 +1380,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1415,7 +1415,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1450,12 +1450,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1476,7 +1476,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -1485,46 +1489,46 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1563,40 +1567,40 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
@@ -1680,12 +1684,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1698,11 +1702,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
@@ -1714,7 +1714,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1758,12 +1762,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1776,7 +1780,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
@@ -1797,12 +1805,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1840,7 +1848,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1883,7 +1891,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1926,7 +1934,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1969,7 +1977,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2012,7 +2020,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2055,12 +2063,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2098,55 +2106,55 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -2184,50 +2192,50 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-15 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M72"/>
+  <dimension ref="A1:M70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -555,18 +555,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -578,12 +582,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -605,12 +609,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -632,7 +636,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -659,7 +663,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -686,12 +690,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -702,7 +706,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -713,7 +721,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -729,7 +737,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -740,7 +752,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -756,7 +768,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -767,7 +783,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -783,7 +799,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -794,12 +814,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -825,12 +845,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -856,27 +876,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -887,7 +907,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -918,27 +938,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -949,7 +969,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -970,7 +990,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
@@ -980,12 +1004,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1050,12 +1074,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1085,32 +1109,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
@@ -1120,12 +1144,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1155,32 +1179,32 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
@@ -1190,12 +1214,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1295,7 +1319,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1330,7 +1354,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1365,7 +1389,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1400,7 +1424,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1435,7 +1459,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1470,46 +1494,46 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1587,46 +1611,46 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1644,11 +1668,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
@@ -1660,85 +1680,89 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1825,50 +1849,50 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1876,42 +1900,42 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1954,7 +1978,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1997,12 +2021,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2083,7 +2107,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2091,90 +2115,90 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2212,12 +2236,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2259,12 +2283,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2306,7 +2330,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2400,12 +2424,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2447,12 +2471,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2478,7 +2502,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
@@ -2494,7 +2522,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Santiago Alvarez Salvado</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2545,12 +2573,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2596,12 +2624,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Santiago Alvarez Salvado</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2647,12 +2675,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2698,12 +2726,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Dídac Petit</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2724,11 +2752,7 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2744,17 +2768,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2775,7 +2803,11 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2791,11 +2823,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2855,12 +2883,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Jordi Lamarca</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2910,12 +2938,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Elisa Volk</t>
+          <t>Jose Manuel Romero</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2965,12 +2993,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3020,12 +3048,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Ricardo Gabriel Castro abad</t>
+          <t>Jordi Lamarca</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3075,12 +3103,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3130,12 +3158,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Jose Manuel Romero</t>
+          <t>Raúl Martínez</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3182,116 +3210,6 @@
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Timan (Nakta) samipour</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Raúl Martínez</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-18 09:22
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -532,18 +532,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -555,7 +559,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -582,7 +586,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -609,12 +613,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -636,22 +640,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -663,12 +671,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -694,7 +702,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -725,12 +733,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -756,12 +764,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -787,27 +795,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -818,12 +826,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -834,12 +842,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -880,12 +888,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -896,7 +904,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>✅</t>
@@ -911,7 +923,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -932,7 +944,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
@@ -942,12 +958,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -977,12 +993,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1012,7 +1028,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1020,24 +1036,24 @@
           <t>Joan</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
@@ -1047,32 +1063,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
@@ -1082,7 +1098,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1152,12 +1168,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1187,7 +1203,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1222,12 +1238,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1257,7 +1273,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1292,7 +1308,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1327,12 +1343,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1362,7 +1378,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1397,7 +1413,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1432,7 +1448,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1467,7 +1483,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1502,7 +1518,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1520,7 +1536,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
@@ -1532,16 +1552,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1619,46 +1635,46 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1676,11 +1692,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
@@ -1692,7 +1704,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1736,7 +1752,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1775,46 +1791,46 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1857,12 +1873,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1900,7 +1916,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1943,12 +1959,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1986,50 +2002,50 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2037,37 +2053,37 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2115,12 +2131,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2158,49 +2174,49 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2252,12 +2268,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2346,7 +2362,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2393,49 +2409,49 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2491,12 +2507,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2542,12 +2558,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2578,27 +2594,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2629,27 +2645,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2695,12 +2711,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Dídac Petit</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2721,7 +2737,11 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J61" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2801,7 +2821,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2809,24 +2829,24 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2856,32 +2876,32 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Timan (Nakta) samipour</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2911,7 +2931,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Timan (Nakta) samipour</t>
+          <t>Raúl Martínez</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2963,61 +2983,6 @@
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Raúl Martínez</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-22 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M65"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -559,12 +559,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -613,7 +613,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -640,28 +640,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -671,12 +671,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -733,12 +733,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -764,12 +764,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -795,27 +795,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -826,12 +826,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -842,7 +842,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>✅</t>
@@ -857,7 +861,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -878,7 +882,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -888,7 +896,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -923,7 +931,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -958,12 +966,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -993,7 +1001,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1028,12 +1036,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1063,32 +1071,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
@@ -1098,12 +1106,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1133,12 +1141,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1168,32 +1176,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
@@ -1203,7 +1211,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1238,12 +1246,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1273,12 +1281,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1308,12 +1316,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1343,7 +1351,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1378,7 +1386,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1413,12 +1421,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1448,12 +1456,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1483,42 +1491,46 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1557,7 +1569,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1596,7 +1608,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1614,11 +1626,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
@@ -1630,7 +1638,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1674,41 +1686,41 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1791,46 +1803,50 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1873,7 +1889,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1881,47 +1897,47 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Xavi Serrallach Pons</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1959,50 +1975,50 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2045,7 +2061,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2053,42 +2069,42 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2174,12 +2190,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2221,7 +2237,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2268,7 +2284,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2315,12 +2331,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2362,7 +2378,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2507,7 +2523,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2558,12 +2574,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2594,27 +2610,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2645,17 +2661,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2711,7 +2727,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2719,24 +2735,24 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2766,12 +2782,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Vanessa Bujaldon Pellicer</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2821,32 +2837,32 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Vanessa Bujaldon Pellicer</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2868,116 +2884,6 @@
         </is>
       </c>
       <c r="M63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Timan (Nakta) samipour</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Raúl Martínez</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M65" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-24 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,12 +559,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -586,7 +586,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -613,12 +613,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -630,7 +630,11 @@
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -640,12 +644,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -656,12 +660,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -702,12 +706,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -764,7 +768,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -931,7 +935,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1071,7 +1075,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1725,7 +1729,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1764,7 +1768,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1846,7 +1850,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1889,7 +1893,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1897,47 +1901,47 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Xavi Serrallach Pons</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1975,93 +1979,93 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2104,50 +2108,50 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2173,7 +2177,11 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
@@ -2190,7 +2198,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2237,12 +2245,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2284,12 +2292,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2331,12 +2339,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2378,79 +2386,79 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2461,23 +2469,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2523,7 +2535,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2574,12 +2586,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2610,47 +2622,47 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2671,17 +2683,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2712,7 +2728,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L60" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2727,32 +2747,32 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2774,116 +2794,6 @@
         </is>
       </c>
       <c r="M61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Marine Fernandez</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Vanessa Bujaldon Pellicer</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-25 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -520,7 +520,11 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -532,7 +536,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -559,7 +563,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -586,7 +590,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -737,12 +741,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -768,27 +772,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -799,28 +803,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -830,7 +838,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -865,7 +873,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -900,7 +908,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -935,7 +943,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -970,7 +978,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1768,132 +1776,136 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1936,7 +1948,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1944,37 +1956,37 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2022,7 +2034,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2030,42 +2042,42 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2108,55 +2120,55 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2198,12 +2210,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2245,12 +2257,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Sara Lucía Ossa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2292,54 +2304,54 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2386,59 +2398,59 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2484,7 +2496,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2535,12 +2547,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2571,22 +2583,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2632,12 +2644,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2645,24 +2661,24 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2692,7 +2708,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2700,24 +2716,24 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>✅</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-01 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -724,12 +724,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -771,12 +771,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -786,27 +786,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -817,28 +817,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -848,7 +848,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -883,7 +883,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -918,12 +918,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -953,7 +953,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -988,7 +988,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1023,12 +1023,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1058,7 +1058,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1093,12 +1093,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1128,12 +1128,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1163,7 +1163,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1198,12 +1198,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1233,12 +1233,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1268,12 +1268,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1303,7 +1303,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1338,7 +1338,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1408,12 +1408,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1478,12 +1478,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1513,32 +1513,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
@@ -1548,32 +1548,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
@@ -1583,71 +1583,79 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1731,90 +1739,90 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1848,12 +1856,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1887,12 +1895,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1926,7 +1934,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1934,42 +1942,42 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2012,7 +2020,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2055,7 +2063,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2098,7 +2106,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2141,50 +2149,50 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2227,12 +2235,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2270,96 +2278,96 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2411,7 +2419,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2429,11 +2437,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
@@ -2447,7 +2451,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2513,7 +2521,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2549,27 +2557,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2615,12 +2623,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Sara Lucía Ossa</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2646,7 +2654,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K61" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2657,16 +2669,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2674,20 +2682,24 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2717,7 +2729,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2725,24 +2737,24 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2772,7 +2784,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2827,12 +2839,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2882,7 +2894,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Roger Defez</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2937,7 +2949,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2989,61 +3001,6 @@
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Gledson Jardim de Vargas</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-06 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -786,12 +786,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -821,7 +821,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -856,7 +856,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -926,7 +926,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -961,12 +961,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -996,12 +996,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1031,12 +1031,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1066,12 +1066,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1101,12 +1101,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1136,7 +1136,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1171,32 +1171,32 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Christopher Rancel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
@@ -1206,12 +1206,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1276,12 +1276,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1311,12 +1311,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1346,7 +1346,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1381,7 +1381,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1451,12 +1451,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1486,12 +1486,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1515,122 +1515,134 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1669,90 +1681,90 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -1825,12 +1837,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1864,12 +1876,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1903,12 +1915,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1942,7 +1954,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1950,37 +1962,37 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2028,50 +2040,50 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2107,52 +2119,60 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2204,54 +2224,54 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2277,12 +2297,12 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
@@ -2298,79 +2318,79 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2381,18 +2401,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2423,7 +2447,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
@@ -2490,7 +2518,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2541,12 +2569,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2592,12 +2620,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2694,32 +2722,32 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2804,7 +2832,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2812,24 +2840,24 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I64" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2859,12 +2887,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-15 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,7 +647,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -658,11 +658,7 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -674,22 +670,18 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -701,22 +693,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -728,22 +716,18 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
@@ -755,7 +739,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -763,16 +747,8 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -786,12 +762,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -802,16 +778,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -821,12 +789,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -837,16 +805,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -856,12 +816,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -872,16 +832,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -891,12 +843,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -907,16 +859,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
@@ -926,32 +870,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
@@ -961,7 +901,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -996,7 +936,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1031,12 +971,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1066,12 +1006,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1101,12 +1041,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1136,12 +1076,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1171,12 +1111,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1206,12 +1146,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1241,32 +1181,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Christopher Rancel</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
@@ -1276,12 +1216,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1311,12 +1251,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1346,51 +1286,47 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1411,11 +1347,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -1424,129 +1356,117 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1580,163 +1500,163 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1775,12 +1695,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -1814,12 +1734,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -1892,12 +1812,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1931,12 +1851,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1970,12 +1890,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -2009,7 +1929,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2017,47 +1937,43 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -2083,11 +1999,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
@@ -2095,50 +2007,46 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2169,11 +2077,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
@@ -2181,59 +2085,55 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Jaume Ràfols Figueras</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2254,11 +2154,7 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
@@ -2275,39 +2171,35 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J53" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2322,80 +2214,84 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2406,26 +2302,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Marcos Molina</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2446,11 +2334,7 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2471,28 +2355,32 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Nizar El Ouarma Sorribas</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2508,26 +2396,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Jaume Ràfols Figueras</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2553,32 +2433,28 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Nizar El Ouarma Sorribas</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2591,11 +2467,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
@@ -2609,7 +2481,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2624,32 +2500,32 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2660,22 +2536,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2721,21 +2597,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2756,11 +2628,7 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2785,32 +2653,32 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Hamza Messaoudi Basaid</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2831,16 +2699,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Marine Fernandez</t>
+          <t>Marcos Molina</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2876,11 +2740,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2895,7 +2755,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2950,12 +2810,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3005,32 +2865,32 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3060,7 +2920,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Roger Defez</t>
+          <t>Marine Fernandez</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3115,12 +2975,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Gledson Jardim de Vargas</t>
+          <t>Hamza Messaoudi Basaid</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3167,6 +3027,281 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Marta Torrente</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Jordi Calmet</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Arnau Rosich Giménez</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Roger Defez</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Gledson Jardim de Vargas</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-23 11:06
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,7 +624,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -658,7 +658,11 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -670,12 +674,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -697,12 +701,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -724,12 +728,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -751,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -767,7 +771,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -778,12 +786,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -794,7 +802,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -836,12 +848,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -867,12 +879,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -902,7 +914,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -937,12 +949,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1007,7 +1019,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1042,12 +1054,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1077,7 +1089,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1112,12 +1124,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1147,12 +1159,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1173,7 +1185,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -1182,12 +1198,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1221,7 +1237,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1299,7 +1315,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1338,7 +1354,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1377,7 +1393,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1416,12 +1432,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1455,7 +1471,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1494,7 +1510,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1533,12 +1549,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1572,7 +1588,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1611,7 +1627,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1650,12 +1666,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1689,7 +1705,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1728,7 +1744,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1806,7 +1822,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1845,7 +1861,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1970,54 +1986,54 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2064,7 +2080,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2111,12 +2127,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -2127,16 +2143,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2152,28 +2160,44 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
@@ -2196,21 +2220,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -2251,12 +2271,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2302,17 +2326,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2338,7 +2366,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K53" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2358,32 +2390,32 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2413,12 +2445,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2468,12 +2500,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2523,7 +2555,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2578,7 +2610,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2633,7 +2665,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2688,12 +2720,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Michela Vistarini</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2743,7 +2775,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2798,7 +2830,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Michela Vistarini</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2853,7 +2885,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Ana Ibáñez</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2908,32 +2940,32 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I64" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3018,12 +3050,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -3073,12 +3105,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-27 09:23
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -509,7 +509,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,7 +647,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -674,12 +674,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -701,7 +701,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -728,12 +728,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -786,12 +786,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -817,7 +817,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -879,7 +879,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -914,7 +914,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -949,7 +949,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -984,7 +984,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1019,7 +1019,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1089,12 +1089,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1124,12 +1124,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1150,7 +1150,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
@@ -1159,12 +1163,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1198,7 +1202,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1237,7 +1241,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1276,7 +1280,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1315,7 +1319,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1354,7 +1358,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1393,12 +1397,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1432,12 +1436,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1471,7 +1475,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1510,7 +1514,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1549,12 +1553,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1588,12 +1592,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1627,12 +1631,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1705,7 +1709,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1744,7 +1748,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1783,7 +1787,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1822,12 +1826,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -1861,59 +1865,75 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1924,31 +1944,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1979,7 +1987,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
     </row>
@@ -2665,12 +2677,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Tania Esther Adrianzen Acero</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2940,12 +2952,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Ángel Herrezuelo Hernández</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -2995,32 +3007,32 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Marta Torrente</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I65" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3050,32 +3062,32 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3105,12 +3117,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-08-06 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M67"/>
+  <dimension ref="A1:M64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,7 +624,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -701,12 +701,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -786,7 +786,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -817,12 +817,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -848,7 +848,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -879,12 +879,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -914,12 +914,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -949,12 +949,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -984,12 +984,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1019,12 +1019,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1054,12 +1054,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1089,12 +1089,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1115,7 +1115,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
@@ -1124,12 +1128,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1163,12 +1167,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1202,12 +1206,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1241,7 +1245,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1280,7 +1284,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1319,12 +1323,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1358,12 +1362,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1397,12 +1401,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1423,12 +1427,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
@@ -1436,12 +1440,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1475,7 +1479,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1514,12 +1518,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1592,7 +1596,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1631,7 +1635,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1670,7 +1674,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1709,12 +1713,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1748,7 +1752,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1779,7 +1783,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
@@ -1787,12 +1795,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -1818,7 +1826,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
@@ -1826,32 +1838,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1862,27 +1862,51 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1893,21 +1917,9 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2002,7 +2014,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2049,12 +2061,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -2065,16 +2077,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2090,28 +2094,44 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
@@ -2134,21 +2154,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -2189,12 +2205,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2240,37 +2260,41 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2300,7 +2324,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2355,12 +2379,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2410,12 +2434,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2465,7 +2489,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2520,7 +2544,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2575,12 +2599,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2630,7 +2654,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Tania Esther Adrianzen Acero</t>
+          <t>Juan Carlos Morales</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2685,32 +2709,32 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Jordi Calmet</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2740,32 +2764,32 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2795,32 +2819,32 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2850,12 +2874,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Ana Ibáñez</t>
+          <t>Marta Torrente</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2905,32 +2929,32 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Ángel Herrezuelo Hernández</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2960,32 +2984,32 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Gledson Jardim de Vargas</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3007,171 +3031,6 @@
         </is>
       </c>
       <c r="M64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Marta Torrente</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Valeria Ontaneda</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Gledson Jardim de Vargas</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-08-07 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -701,12 +701,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -786,7 +786,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -817,12 +817,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -848,7 +848,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -879,7 +879,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -914,12 +914,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -949,12 +949,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -984,7 +984,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1019,12 +1019,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1054,12 +1054,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1128,12 +1128,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1206,7 +1206,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1284,12 +1284,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1323,7 +1323,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1362,12 +1362,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1401,12 +1401,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1427,12 +1427,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
@@ -1440,7 +1440,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1479,7 +1479,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1518,7 +1518,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1557,12 +1557,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1583,12 +1583,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -1596,12 +1596,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1635,7 +1635,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1674,7 +1674,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1713,12 +1713,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1795,32 +1795,20 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1831,27 +1819,51 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1862,31 +1874,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1924,12 +1924,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1960,19 +1960,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -2014,12 +2018,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -2544,7 +2548,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2929,7 +2933,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-08-13 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -674,12 +674,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -690,7 +690,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -701,12 +705,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -717,7 +721,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -728,12 +736,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -744,7 +752,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -755,12 +767,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -786,12 +798,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -807,7 +819,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -817,12 +833,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -838,7 +854,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -848,12 +868,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -869,7 +889,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -879,7 +903,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -914,7 +938,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -949,12 +973,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-08-14 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -1152,12 +1152,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1191,7 +1191,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1269,12 +1269,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1308,12 +1308,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1347,12 +1347,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1425,12 +1425,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1464,12 +1464,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1503,7 +1503,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1542,12 +1542,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1568,12 +1568,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
@@ -1581,12 +1581,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1607,12 +1607,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -1620,12 +1620,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1659,7 +1659,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1698,12 +1698,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1737,12 +1737,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1768,7 +1768,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
@@ -1776,7 +1780,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-08-17 13:53
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -624,7 +624,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -635,7 +635,11 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -647,12 +651,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -674,7 +678,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -705,12 +709,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -736,7 +740,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -767,12 +771,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -798,12 +802,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -833,7 +837,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -868,7 +872,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -903,12 +907,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -938,12 +942,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -973,12 +977,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1008,7 +1012,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Yonadxandi Manriquez Ledezma</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1043,7 +1047,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1078,7 +1082,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1104,7 +1108,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
@@ -1113,12 +1121,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1152,7 +1160,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1191,7 +1199,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1230,7 +1238,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1269,12 +1277,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1308,7 +1316,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1347,12 +1355,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1386,7 +1394,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1425,12 +1433,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1464,7 +1472,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1503,7 +1511,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1542,12 +1550,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1568,12 +1576,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
@@ -1581,7 +1589,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1620,7 +1628,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1659,12 +1667,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1685,12 +1693,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
@@ -1698,12 +1706,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1737,12 +1745,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1866,12 +1874,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-08-25 09:33
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -1121,12 +1121,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1160,7 +1160,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1199,7 +1199,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1238,7 +1238,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1316,12 +1316,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1355,12 +1355,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1394,12 +1394,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1433,12 +1433,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1472,12 +1472,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1511,7 +1511,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1550,7 +1550,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1589,12 +1589,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1615,12 +1615,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -1628,7 +1628,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1667,12 +1667,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1693,7 +1693,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1706,7 +1710,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1737,7 +1741,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
@@ -1745,12 +1753,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1788,12 +1796,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -1831,20 +1839,32 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1855,51 +1875,27 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1910,19 +1906,31 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1953,19 +1961,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>

</xml_diff>